<commit_message>
lots of change; finished ai reviews; modified scripts
</commit_message>
<xml_diff>
--- a/data/vendor-search/results_all_alarms.xlsx
+++ b/data/vendor-search/results_all_alarms.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G104"/>
+  <dimension ref="A1:H104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,11 @@
           <t>cpe_strings</t>
         </is>
       </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>matched_terms</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -472,8 +477,10 @@
       <c r="D2" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E2" t="n">
-        <v>3</v>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -483,6 +490,11 @@
       <c r="G2" t="inlineStr">
         <is>
           <t>cpe:2.3:o:netgear:arlo_base_station_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:netgear:vmb30x0:-:*:*:*:*:*:*:*|cpe:2.3:h:netgear:vmk3xx0:-:*:*:*:*:*:*:*|cpe:2.3:h:netgear:vms3xx0:-:*:*:*:*:*:*:*|cpe:2.3:o:netgear:arlo_q_camera_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:netgear:vmc3040:-:*:*:*:*:*:*:*|cpe:2.3:o:netgear:arlo_q_plus_camera_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:netgear:vmc3040s:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>arlo base station</t>
         </is>
       </c>
     </row>
@@ -505,8 +517,10 @@
       <c r="D3" t="n">
         <v>8.1</v>
       </c>
-      <c r="E3" t="n">
-        <v>3</v>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -516,6 +530,11 @@
       <c r="G3" t="inlineStr">
         <is>
           <t>cpe:2.3:o:netgear:arlo_base_station_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:netgear:vmb30x0:-:*:*:*:*:*:*:*|cpe:2.3:h:netgear:vmk3xx0:-:*:*:*:*:*:*:*|cpe:2.3:h:netgear:vms3xx0:-:*:*:*:*:*:*:*|cpe:2.3:o:netgear:arlo_q_camera_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:netgear:vmc3040:-:*:*:*:*:*:*:*|cpe:2.3:o:netgear:arlo_q_plus_camera_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:netgear:vmc3040s:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>arlo base station</t>
         </is>
       </c>
     </row>
@@ -538,8 +557,10 @@
       <c r="D4" t="n">
         <v>4.3</v>
       </c>
-      <c r="E4" t="n">
-        <v>3</v>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -549,6 +570,11 @@
       <c r="G4" t="inlineStr">
         <is>
           <t>cpe:2.3:o:simplisafe:u9k-es1000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:simplisafe:u9k-es1000:-:*:*:*:*:*:*:*|cpe:2.3:o:simplisafe:u9k-kr1_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:simplisafe:u9k-kr1:-:*:*:*:*:*:*:*|cpe:2.3:o:simplisafe:u9k-ms1000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:simplisafe:u9k-ms1000:-:*:*:*:*:*:*:*|cpe:2.3:o:simplisafe:u9k-wt1000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:simplisafe:u9k-wt1000:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>simplisafe</t>
         </is>
       </c>
     </row>
@@ -571,8 +597,10 @@
       <c r="D5" t="n">
         <v>4.6</v>
       </c>
-      <c r="E5" t="n">
-        <v>3</v>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr">
@@ -580,6 +608,11 @@
           <t>cpe:2.3:o:simplisafe:u9k-bs1000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:simplisafe:u9k-bs1000:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>simplisafe</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -600,8 +633,10 @@
       <c r="D6" t="n">
         <v>4.6</v>
       </c>
-      <c r="E6" t="n">
-        <v>3</v>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr">
@@ -609,6 +644,11 @@
           <t>cpe:2.3:o:simplisafe:u9k-bs1000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:simplisafe:u9k-bs1000:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>simplisafe</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -629,8 +669,10 @@
       <c r="D7" t="n">
         <v>6.6</v>
       </c>
-      <c r="E7" t="n">
-        <v>3</v>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -640,6 +682,11 @@
       <c r="G7" t="inlineStr">
         <is>
           <t>cpe:2.3:o:simplisafe:u9k-kp1000_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:simplisafe:u9k-kp1000:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>simplisafe</t>
         </is>
       </c>
     </row>
@@ -662,8 +709,10 @@
       <c r="D8" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E8" t="n">
-        <v>3</v>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
@@ -673,6 +722,11 @@
       <c r="G8" t="inlineStr">
         <is>
           <t>cpe:2.3:a:idera:uptime_infrastructure_monitor:7.4.0:*:*:*:*:*:*:*|cpe:2.3:a:idera:uptime_infrastructure_monitor:7.5.0:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>monitoring station</t>
         </is>
       </c>
     </row>
@@ -695,8 +749,10 @@
       <c r="D9" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E9" t="n">
-        <v>3.1</v>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -706,6 +762,11 @@
       <c r="G9" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -728,8 +789,10 @@
       <c r="D10" t="n">
         <v>9.9</v>
       </c>
-      <c r="E10" t="n">
-        <v>3.1</v>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -739,6 +802,11 @@
       <c r="G10" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -761,8 +829,10 @@
       <c r="D11" t="n">
         <v>7.5</v>
       </c>
-      <c r="E11" t="n">
-        <v>3.1</v>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
@@ -772,6 +842,11 @@
       <c r="G11" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -794,8 +869,10 @@
       <c r="D12" t="n">
         <v>5.9</v>
       </c>
-      <c r="E12" t="n">
-        <v>3</v>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -805,6 +882,11 @@
       <c r="G12" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -827,8 +909,10 @@
       <c r="D13" t="n">
         <v>5.5</v>
       </c>
-      <c r="E13" t="n">
-        <v>3.1</v>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -838,6 +922,11 @@
       <c r="G13" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -860,8 +949,10 @@
       <c r="D14" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E14" t="n">
-        <v>3.1</v>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -871,6 +962,11 @@
       <c r="G14" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -893,8 +989,10 @@
       <c r="D15" t="n">
         <v>7.5</v>
       </c>
-      <c r="E15" t="n">
-        <v>3.1</v>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -904,6 +1002,11 @@
       <c r="G15" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -926,8 +1029,10 @@
       <c r="D16" t="n">
         <v>7.8</v>
       </c>
-      <c r="E16" t="n">
-        <v>3.1</v>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
@@ -937,6 +1042,11 @@
       <c r="G16" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -959,8 +1069,10 @@
       <c r="D17" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E17" t="n">
-        <v>3.1</v>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
@@ -970,6 +1082,11 @@
       <c r="G17" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -992,8 +1109,10 @@
       <c r="D18" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E18" t="n">
-        <v>3.1</v>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
@@ -1003,6 +1122,11 @@
       <c r="G18" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -1025,8 +1149,10 @@
       <c r="D19" t="n">
         <v>9.9</v>
       </c>
-      <c r="E19" t="n">
-        <v>3.1</v>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
@@ -1036,6 +1162,11 @@
       <c r="G19" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -1058,8 +1189,10 @@
       <c r="D20" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E20" t="n">
-        <v>3.1</v>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1069,6 +1202,11 @@
       <c r="G20" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -1091,8 +1229,10 @@
       <c r="D21" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E21" t="n">
-        <v>3.1</v>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
@@ -1102,6 +1242,11 @@
       <c r="G21" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -1124,8 +1269,10 @@
       <c r="D22" t="n">
         <v>9.9</v>
       </c>
-      <c r="E22" t="n">
-        <v>3.1</v>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
@@ -1135,6 +1282,11 @@
       <c r="G22" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -1157,8 +1309,10 @@
       <c r="D23" t="n">
         <v>9.9</v>
       </c>
-      <c r="E23" t="n">
-        <v>3.1</v>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
@@ -1168,6 +1322,11 @@
       <c r="G23" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -1190,8 +1349,10 @@
       <c r="D24" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E24" t="n">
-        <v>3.1</v>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
@@ -1201,6 +1362,11 @@
       <c r="G24" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -1223,8 +1389,10 @@
       <c r="D25" t="n">
         <v>9.9</v>
       </c>
-      <c r="E25" t="n">
-        <v>3.1</v>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F25" t="inlineStr">
         <is>
@@ -1234,6 +1402,11 @@
       <c r="G25" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -1256,8 +1429,10 @@
       <c r="D26" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E26" t="n">
-        <v>3.1</v>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F26" t="inlineStr">
         <is>
@@ -1267,6 +1442,11 @@
       <c r="G26" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -1289,8 +1469,10 @@
       <c r="D27" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="E27" t="n">
-        <v>3.1</v>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F27" t="inlineStr">
         <is>
@@ -1300,6 +1482,11 @@
       <c r="G27" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -1322,8 +1509,10 @@
       <c r="D28" t="n">
         <v>6.7</v>
       </c>
-      <c r="E28" t="n">
-        <v>3.1</v>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F28" t="inlineStr">
         <is>
@@ -1333,6 +1522,11 @@
       <c r="G28" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -1355,8 +1549,10 @@
       <c r="D29" t="n">
         <v>7.8</v>
       </c>
-      <c r="E29" t="n">
-        <v>3.1</v>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
@@ -1366,6 +1562,11 @@
       <c r="G29" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -1388,8 +1589,10 @@
       <c r="D30" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="E30" t="n">
-        <v>3.1</v>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F30" t="inlineStr">
         <is>
@@ -1399,6 +1602,11 @@
       <c r="G30" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -1421,8 +1629,10 @@
       <c r="D31" t="n">
         <v>7.2</v>
       </c>
-      <c r="E31" t="n">
-        <v>3</v>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
@@ -1432,6 +1642,11 @@
       <c r="G31" t="inlineStr">
         <is>
           <t>cpe:2.3:o:alarm:adc-v522ir_firmware:0100b9:*:*:*:*:*:*:*|cpe:2.3:h:alarm:adc-v522ir:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>alarm.com</t>
         </is>
       </c>
     </row>
@@ -1454,8 +1669,10 @@
       <c r="D32" t="n">
         <v>7.8</v>
       </c>
-      <c r="E32" t="n">
-        <v>3</v>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -1465,6 +1682,11 @@
       <c r="G32" t="inlineStr">
         <is>
           <t>cpe:2.3:o:alarm:adc-v522ir_firmware:0100b9:*:*:*:*:*:*:*|cpe:2.3:h:alarm:adc-v522ir:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>alarm.com</t>
         </is>
       </c>
     </row>
@@ -1487,8 +1709,10 @@
       <c r="D33" t="n">
         <v>4.6</v>
       </c>
-      <c r="E33" t="n">
-        <v>3.1</v>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
@@ -1498,6 +1722,11 @@
       <c r="G33" t="inlineStr">
         <is>
           <t>cpe:2.3:o:simplisafe:ss3_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:simplisafe:ss3:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>simplisafe</t>
         </is>
       </c>
     </row>
@@ -1520,8 +1749,10 @@
       <c r="D34" t="n">
         <v>10</v>
       </c>
-      <c r="E34" t="n">
-        <v>3.1</v>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1531,6 +1762,11 @@
       <c r="G34" t="inlineStr">
         <is>
           <t>cpe:2.3:o:gehealthcare:apexpro_telemetry_server_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:apexpro_telemetry_server:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mai700_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_central_station_mai700:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mas700_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_central_station_mas700:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100d_firmware:4.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100d_firmware:5.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:clinical_information_center_mp100d:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100r_firmware:4.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100r_firmware:5.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:clinical_information_center_mp100r:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_telemetry_server_mp100r_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_telemetry_server_mp100r_firmware:4.3:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_telemetry_server_mp100r:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>central station</t>
         </is>
       </c>
     </row>
@@ -1553,8 +1789,10 @@
       <c r="D35" t="n">
         <v>10</v>
       </c>
-      <c r="E35" t="n">
-        <v>3.1</v>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F35" t="inlineStr">
         <is>
@@ -1564,6 +1802,11 @@
       <c r="G35" t="inlineStr">
         <is>
           <t>cpe:2.3:o:gehealthcare:apexpro_telemetry_server_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:apexpro_telemetry_server_firmware:4.3:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:apexpro_telemetry_server:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_b450_monitor_firmware:2.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_b450_monitor:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_b650_monitor_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_b650_monitor_firmware:2.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_b650_monitor:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_b850_monitor_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_b850_monitor_firmware:2.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_b850_monitor:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mai700_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mai700_firmware:2.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_central_station_mai700:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mas700_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mas700_firmware:2.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_central_station_mas700:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100d_firmware:4.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100d_firmware:5.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:clinical_information_center_mp100d:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100r_firmware:4.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100r_firmware:5.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:clinical_information_center_mp100r:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_telemetry_server_mp100r_firmware:*:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_telemetry_server_mp100r_firmware:4.3:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_telemetry_server_mp100r:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>central station</t>
         </is>
       </c>
     </row>
@@ -1586,8 +1829,10 @@
       <c r="D36" t="n">
         <v>10</v>
       </c>
-      <c r="E36" t="n">
-        <v>3.1</v>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F36" t="inlineStr">
         <is>
@@ -1597,6 +1842,11 @@
       <c r="G36" t="inlineStr">
         <is>
           <t>cpe:2.3:o:gehealthcare:apexpro_telemetry_server_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:apexpro_telemetry_server:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mai700_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_central_station_mai700:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mas700_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_central_station_mas700:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100d_firmware:4.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100d_firmware:5.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:clinical_information_center_mp100d:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100r_firmware:4.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100r_firmware:5.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:clinical_information_center_mp100r:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_telemetry_server_mp100r_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_telemetry_server_mp100r:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>central station</t>
         </is>
       </c>
     </row>
@@ -1619,8 +1869,10 @@
       <c r="D37" t="n">
         <v>8.6</v>
       </c>
-      <c r="E37" t="n">
-        <v>3.1</v>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -1630,6 +1882,11 @@
       <c r="G37" t="inlineStr">
         <is>
           <t>cpe:2.3:o:gehealthcare:apexpro_telemetry_server_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:apexpro_telemetry_server:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mai700_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mai700_firmware:2.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_central_station_mai700:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mas700_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mas700_firmware:2.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_central_station_mas700:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100d_firmware:4.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100d_firmware:5.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:clinical_information_center_mp100d:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100r_firmware:4.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100r_firmware:5.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:clinical_information_center_mp100r:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_telemetry_server_mp100r_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_telemetry_server_mp100r:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>central station</t>
         </is>
       </c>
     </row>
@@ -1652,8 +1909,10 @@
       <c r="D38" t="n">
         <v>9.9</v>
       </c>
-      <c r="E38" t="n">
-        <v>3.1</v>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F38" t="inlineStr">
         <is>
@@ -1663,6 +1922,11 @@
       <c r="G38" t="inlineStr">
         <is>
           <t>cpe:2.3:o:gehealthcare:apexpro_telemetry_server_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:apexpro_telemetry_server:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_b450_monitor_firmware:2.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_b450_monitor:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_b650_monitor_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_b650_monitor_firmware:2.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_b650_monitor:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_b850_monitor_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_b850_monitor_firmware:2.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_b850_monitor:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mai700_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_central_station_mai700:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mas700_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_central_station_mas700:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100d_firmware:4.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100d_firmware:5.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:clinical_information_center_mp100d:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100r_firmware:4.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100r_firmware:5.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:clinical_information_center_mp100r:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_telemetry_server_mp100r_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_telemetry_server_mp100r:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>central station</t>
         </is>
       </c>
     </row>
@@ -1685,8 +1949,10 @@
       <c r="D39" t="n">
         <v>10</v>
       </c>
-      <c r="E39" t="n">
-        <v>3.1</v>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
@@ -1696,6 +1962,11 @@
       <c r="G39" t="inlineStr">
         <is>
           <t>cpe:2.3:o:gehealthcare:apexpro_telemetry_server_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:apexpro_telemetry_server:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mai700_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_central_station_mai700:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_central_station_mas700_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_central_station_mas700:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100d_firmware:4.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100d_firmware:5.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:clinical_information_center_mp100d:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100r_firmware:4.0:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:clinical_information_center_mp100r_firmware:5.0:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:clinical_information_center_mp100r:-:*:*:*:*:*:*:*|cpe:2.3:o:gehealthcare:carescape_telemetry_server_mp100r_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:gehealthcare:carescape_telemetry_server_mp100r:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>central station</t>
         </is>
       </c>
     </row>
@@ -1718,8 +1989,10 @@
       <c r="D40" t="n">
         <v>10</v>
       </c>
-      <c r="E40" t="n">
-        <v>3.1</v>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
@@ -1729,6 +2002,11 @@
       <c r="G40" t="inlineStr">
         <is>
           <t>cpe:2.3:o:anker:eufy_homebase_2_firmware:2.1.6.9h:*:*:*:*:*:*:*|cpe:2.3:h:anker:eufy_homebase_2:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>eufy homebase</t>
         </is>
       </c>
     </row>
@@ -1751,8 +2029,10 @@
       <c r="D41" t="n">
         <v>9</v>
       </c>
-      <c r="E41" t="n">
-        <v>3.1</v>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
@@ -1762,6 +2042,11 @@
       <c r="G41" t="inlineStr">
         <is>
           <t>cpe:2.3:o:anker:eufy_homebase_2_firmware:2.1.6.9h:*:*:*:*:*:*:*|cpe:2.3:h:anker:eufy_homebase_2:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>eufy homebase</t>
         </is>
       </c>
     </row>
@@ -1784,8 +2069,10 @@
       <c r="D42" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E42" t="n">
-        <v>3.1</v>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F42" t="inlineStr">
         <is>
@@ -1795,6 +2082,11 @@
       <c r="G42" t="inlineStr">
         <is>
           <t>cpe:2.3:o:anker:eufy_homebase_2_firmware:2.1.8.5h:*:*:*:*:*:*:*|cpe:2.3:h:anker:eufy_homebase_2:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>eufy homebase</t>
         </is>
       </c>
     </row>
@@ -1817,8 +2109,10 @@
       <c r="D43" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E43" t="n">
-        <v>3.1</v>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
@@ -1828,6 +2122,11 @@
       <c r="G43" t="inlineStr">
         <is>
           <t>cpe:2.3:o:anker:eufy_homebase_2_firmware:2.1.8.5h:*:*:*:*:*:*:*|cpe:2.3:h:anker:eufy_homebase_2:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>eufy homebase</t>
         </is>
       </c>
     </row>
@@ -1850,8 +2149,10 @@
       <c r="D44" t="n">
         <v>6.5</v>
       </c>
-      <c r="E44" t="n">
-        <v>3.1</v>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F44" t="inlineStr">
         <is>
@@ -1861,6 +2162,11 @@
       <c r="G44" t="inlineStr">
         <is>
           <t>cpe:2.3:o:anker:eufy_homebase_2_firmware:2.1.8.5h:*:*:*:*:*:*:*|cpe:2.3:h:anker:eufy_homebase_2:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>eufy homebase</t>
         </is>
       </c>
     </row>
@@ -1883,8 +2189,10 @@
       <c r="D45" t="n">
         <v>10</v>
       </c>
-      <c r="E45" t="n">
-        <v>3.1</v>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -1894,6 +2202,11 @@
       <c r="G45" t="inlineStr">
         <is>
           <t>cpe:2.3:o:getnexx:nxal-100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxal-100:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxg-100b_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxg-100b:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxpg-100w_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxpg-100w:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxg-200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxg-200:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>nexx</t>
         </is>
       </c>
     </row>
@@ -1916,8 +2229,10 @@
       <c r="D46" t="n">
         <v>6.5</v>
       </c>
-      <c r="E46" t="n">
-        <v>3.1</v>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
@@ -1927,6 +2242,11 @@
       <c r="G46" t="inlineStr">
         <is>
           <t>cpe:2.3:o:getnexx:nxal-100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxal-100:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxg-100b_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxg-100b:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxpg-100w_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxpg-100w:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxg-200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxg-200:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>nexx</t>
         </is>
       </c>
     </row>
@@ -1949,8 +2269,10 @@
       <c r="D47" t="n">
         <v>7.1</v>
       </c>
-      <c r="E47" t="n">
-        <v>3.1</v>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -1960,6 +2282,11 @@
       <c r="G47" t="inlineStr">
         <is>
           <t>cpe:2.3:o:getnexx:nxal-100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxal-100:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxg-100b_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxg-100b:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxpg-100w_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxpg-100w:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxg-200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxg-200:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>nexx</t>
         </is>
       </c>
     </row>
@@ -1982,8 +2309,10 @@
       <c r="D48" t="n">
         <v>5.3</v>
       </c>
-      <c r="E48" t="n">
-        <v>3.1</v>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr">
@@ -1991,6 +2320,11 @@
           <t>cpe:2.3:o:getnexx:nxal-100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxal-100:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxg-100b_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxg-100b:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxpg-100w_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxpg-100w:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxg-200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxg-200:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>nexx</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2011,8 +2345,10 @@
       <c r="D49" t="n">
         <v>4.3</v>
       </c>
-      <c r="E49" t="n">
-        <v>3.1</v>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2022,6 +2358,11 @@
       <c r="G49" t="inlineStr">
         <is>
           <t>cpe:2.3:o:getnexx:nxal-100_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxal-100:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxg-100b_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxg-100b:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxpg-100w_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxpg-100w:-:*:*:*:*:*:*:*|cpe:2.3:o:getnexx:nxg-200_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:getnexx:nxg-200:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>nexx</t>
         </is>
       </c>
     </row>
@@ -2044,8 +2385,10 @@
       <c r="D50" t="n">
         <v>7.5</v>
       </c>
-      <c r="E50" t="n">
-        <v>3.1</v>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F50" t="inlineStr">
         <is>
@@ -2055,6 +2398,11 @@
       <c r="G50" t="inlineStr">
         <is>
           <t>cpe:2.3:o:blitzwolf:bw-is22_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:h:blitzwolf:bw-is22:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>security alarm</t>
         </is>
       </c>
     </row>
@@ -2077,8 +2425,10 @@
       <c r="D51" t="n">
         <v>7.5</v>
       </c>
-      <c r="E51" t="n">
-        <v>3.1</v>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F51" t="inlineStr">
         <is>
@@ -2088,6 +2438,11 @@
       <c r="G51" t="inlineStr">
         <is>
           <t>cpe:2.3:o:agshome_smart_alarm_project:agshome_smart_alarm_firmware:1.0:*:*:*:*:*:*:*|cpe:2.3:h:agshome_smart_alarm_project:agshome_smart_alarm:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>agshome|smart alarm</t>
         </is>
       </c>
     </row>
@@ -2110,8 +2465,10 @@
       <c r="D52" t="n">
         <v>8.199999999999999</v>
       </c>
-      <c r="E52" t="n">
-        <v>3.1</v>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F52" t="inlineStr">
         <is>
@@ -2121,6 +2478,11 @@
       <c r="G52" t="inlineStr">
         <is>
           <t>cpe:2.3:o:eufy:homebase_2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:eufy:homebase_2:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>eufy homebase</t>
         </is>
       </c>
     </row>
@@ -2143,8 +2505,10 @@
       <c r="D53" t="n">
         <v>3.5</v>
       </c>
-      <c r="E53" t="n">
-        <v>2</v>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -2154,6 +2518,11 @@
       <c r="G53" t="inlineStr">
         <is>
           <t>cpe:2.3:o:dlink:dsl-2730b_firmware:ge_1.01:*:*:*:*:*:*:*|cpe:2.3:h:dlink:dsl-2730b:c1:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>security panel</t>
         </is>
       </c>
     </row>
@@ -2176,8 +2545,10 @@
       <c r="D54" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="E54" t="n">
-        <v>2</v>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F54" t="inlineStr">
         <is>
@@ -2187,6 +2558,11 @@
       <c r="G54" t="inlineStr">
         <is>
           <t>cpe:2.3:a:qolsys:iq_panel:*:*:*:*:*:android:*:*</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>qolsys|qolsys iq panel</t>
         </is>
       </c>
     </row>
@@ -2209,8 +2585,10 @@
       <c r="D55" t="n">
         <v>9.300000000000001</v>
       </c>
-      <c r="E55" t="n">
-        <v>2</v>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>2.0</t>
+        </is>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -2220,6 +2598,11 @@
       <c r="G55" t="inlineStr">
         <is>
           <t>cpe:2.3:a:qolsys:iq_panel:*:*:*:*:*:android:*:*</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>qolsys|qolsys iq panel</t>
         </is>
       </c>
     </row>
@@ -2242,8 +2625,10 @@
       <c r="D56" t="n">
         <v>6.5</v>
       </c>
-      <c r="E56" t="n">
-        <v>3</v>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F56" t="inlineStr">
         <is>
@@ -2253,6 +2638,11 @@
       <c r="G56" t="inlineStr">
         <is>
           <t>cpe:2.3:o:philips:intellivue_mx40_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:philips:intellivue_mx40:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>monitoring station</t>
         </is>
       </c>
     </row>
@@ -2275,8 +2665,10 @@
       <c r="D57" t="n">
         <v>6.5</v>
       </c>
-      <c r="E57" t="n">
-        <v>3</v>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F57" t="inlineStr">
         <is>
@@ -2286,6 +2678,11 @@
       <c r="G57" t="inlineStr">
         <is>
           <t>cpe:2.3:o:philips:intellivue_mx40_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:philips:intellivue_mx40:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>monitoring station</t>
         </is>
       </c>
     </row>
@@ -2308,8 +2705,10 @@
       <c r="D58" t="n">
         <v>9.9</v>
       </c>
-      <c r="E58" t="n">
-        <v>3.1</v>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
@@ -2319,6 +2718,11 @@
       <c r="G58" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2341,8 +2745,10 @@
       <c r="D59" t="n">
         <v>9.9</v>
       </c>
-      <c r="E59" t="n">
-        <v>3.1</v>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -2352,6 +2758,11 @@
       <c r="G59" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2374,8 +2785,10 @@
       <c r="D60" t="n">
         <v>9.9</v>
       </c>
-      <c r="E60" t="n">
-        <v>3.1</v>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
@@ -2385,6 +2798,11 @@
       <c r="G60" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2407,8 +2825,10 @@
       <c r="D61" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E61" t="n">
-        <v>3.1</v>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -2418,6 +2838,11 @@
       <c r="G61" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2440,8 +2865,10 @@
       <c r="D62" t="n">
         <v>9.9</v>
       </c>
-      <c r="E62" t="n">
-        <v>3.1</v>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
@@ -2451,6 +2878,11 @@
       <c r="G62" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2473,8 +2905,10 @@
       <c r="D63" t="n">
         <v>9.9</v>
       </c>
-      <c r="E63" t="n">
-        <v>3.1</v>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
@@ -2484,6 +2918,11 @@
       <c r="G63" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2506,8 +2945,10 @@
       <c r="D64" t="n">
         <v>9.9</v>
       </c>
-      <c r="E64" t="n">
-        <v>3.1</v>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -2517,6 +2958,11 @@
       <c r="G64" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2539,8 +2985,10 @@
       <c r="D65" t="n">
         <v>9.9</v>
       </c>
-      <c r="E65" t="n">
-        <v>3.1</v>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F65" t="inlineStr">
         <is>
@@ -2550,6 +2998,11 @@
       <c r="G65" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2572,8 +3025,10 @@
       <c r="D66" t="n">
         <v>9.9</v>
       </c>
-      <c r="E66" t="n">
-        <v>3.1</v>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
@@ -2583,6 +3038,11 @@
       <c r="G66" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2605,8 +3065,10 @@
       <c r="D67" t="n">
         <v>9.9</v>
       </c>
-      <c r="E67" t="n">
-        <v>3</v>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F67" t="inlineStr">
         <is>
@@ -2616,6 +3078,11 @@
       <c r="G67" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2638,8 +3105,10 @@
       <c r="D68" t="n">
         <v>7.8</v>
       </c>
-      <c r="E68" t="n">
-        <v>3.1</v>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -2649,6 +3118,11 @@
       <c r="G68" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2671,8 +3145,10 @@
       <c r="D69" t="n">
         <v>9.9</v>
       </c>
-      <c r="E69" t="n">
-        <v>3.1</v>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
@@ -2682,6 +3158,11 @@
       <c r="G69" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2704,8 +3185,10 @@
       <c r="D70" t="n">
         <v>9.9</v>
       </c>
-      <c r="E70" t="n">
-        <v>3.1</v>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
@@ -2715,6 +3198,11 @@
       <c r="G70" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2737,8 +3225,10 @@
       <c r="D71" t="n">
         <v>9.9</v>
       </c>
-      <c r="E71" t="n">
-        <v>3.1</v>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F71" t="inlineStr">
         <is>
@@ -2748,6 +3238,11 @@
       <c r="G71" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2770,8 +3265,10 @@
       <c r="D72" t="n">
         <v>9.9</v>
       </c>
-      <c r="E72" t="n">
-        <v>3.1</v>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F72" t="inlineStr">
         <is>
@@ -2781,6 +3278,11 @@
       <c r="G72" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2803,8 +3305,10 @@
       <c r="D73" t="n">
         <v>8.6</v>
       </c>
-      <c r="E73" t="n">
-        <v>3.1</v>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F73" t="inlineStr">
         <is>
@@ -2814,6 +3318,11 @@
       <c r="G73" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2836,8 +3345,10 @@
       <c r="D74" t="n">
         <v>10</v>
       </c>
-      <c r="E74" t="n">
-        <v>3.1</v>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F74" t="inlineStr">
         <is>
@@ -2847,6 +3358,11 @@
       <c r="G74" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2869,8 +3385,10 @@
       <c r="D75" t="n">
         <v>8.6</v>
       </c>
-      <c r="E75" t="n">
-        <v>3.1</v>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F75" t="inlineStr">
         <is>
@@ -2880,6 +3398,11 @@
       <c r="G75" t="inlineStr">
         <is>
           <t>cpe:2.3:o:samsung:sth-eth-250_firmware:0.20.17:*:*:*:*:*:*:*|cpe:2.3:h:samsung:sth-eth-250:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>samsung smartthings hub</t>
         </is>
       </c>
     </row>
@@ -2902,8 +3425,10 @@
       <c r="D76" t="n">
         <v>6.5</v>
       </c>
-      <c r="E76" t="n">
-        <v>3</v>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F76" t="inlineStr">
         <is>
@@ -2913,6 +3438,11 @@
       <c r="G76" t="inlineStr">
         <is>
           <t>cpe:2.3:o:abus:secvest_wireless_alarm_system_fuaa50000_firmware:3.01.01:*:*:*:*:*:*:*|cpe:2.3:h:abus:secvest_wireless_alarm_system_fuaa50000:-:*:*:*:*:*:*:*|cpe:2.3:o:abus:secvest_wireless_remote_control_fube50014_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:abus:secvest_wireless_remote_control_fube50014:-:*:*:*:*:*:*:*|cpe:2.3:o:abus:secvest_wireless_remote_control_fube50015_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:abus:secvest_wireless_remote_control_fube50015:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>wireless alarm system</t>
         </is>
       </c>
     </row>
@@ -2935,8 +3465,10 @@
       <c r="D77" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E77" t="n">
-        <v>3</v>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F77" t="inlineStr">
         <is>
@@ -2946,6 +3478,11 @@
       <c r="G77" t="inlineStr">
         <is>
           <t>cpe:2.3:o:abus:secvest_wireless_alarm_system_fuaa50000_firmware:3.01.01:*:*:*:*:*:*:*|cpe:2.3:h:abus:secvest_wireless_alarm_system_fuaa50000:-:*:*:*:*:*:*:*|cpe:2.3:o:abus:secvest_wireless_remote_control_fube50014_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:abus:secvest_wireless_remote_control_fube50014:-:*:*:*:*:*:*:*|cpe:2.3:o:abus:secvest_wireless_remote_control_fube50015_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:abus:secvest_wireless_remote_control_fube50015:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>wireless alarm system</t>
         </is>
       </c>
     </row>
@@ -2968,8 +3505,10 @@
       <c r="D78" t="n">
         <v>7.5</v>
       </c>
-      <c r="E78" t="n">
-        <v>3</v>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F78" t="inlineStr">
         <is>
@@ -2979,6 +3518,11 @@
       <c r="G78" t="inlineStr">
         <is>
           <t>cpe:2.3:o:abus:secvest_wireless_alarm_system_fuaa50000_firmware:3.01.01:*:*:*:*:*:*:*|cpe:2.3:h:abus:secvest_wireless_alarm_system_fuaa50000:-:*:*:*:*:*:*:*|cpe:2.3:o:abus:secvest_wireless_remote_control_fube50014_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:abus:secvest_wireless_remote_control_fube50014:-:*:*:*:*:*:*:*|cpe:2.3:o:abus:secvest_wireless_remote_control_fube50015_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:abus:secvest_wireless_remote_control_fube50015:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>wireless alarm system</t>
         </is>
       </c>
     </row>
@@ -3001,8 +3545,10 @@
       <c r="D79" t="n">
         <v>8.1</v>
       </c>
-      <c r="E79" t="n">
-        <v>3</v>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
@@ -3012,6 +3558,11 @@
       <c r="G79" t="inlineStr">
         <is>
           <t>cpe:2.3:o:abus:secvest_wireless_alarm_system_fuaa50000_firmware:3.01.01:*:*:*:*:*:*:*|cpe:2.3:h:abus:secvest_wireless_alarm_system_fuaa50000:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>wireless alarm system</t>
         </is>
       </c>
     </row>
@@ -3034,8 +3585,10 @@
       <c r="D80" t="n">
         <v>7.5</v>
       </c>
-      <c r="E80" t="n">
-        <v>3</v>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>3.0</t>
+        </is>
       </c>
       <c r="F80" t="inlineStr">
         <is>
@@ -3045,6 +3598,11 @@
       <c r="G80" t="inlineStr">
         <is>
           <t>cpe:2.3:o:abus:secvest_wireless_alarm_system_fuaa50000_firmware:3.01.01:*:*:*:*:*:*:*|cpe:2.3:h:abus:secvest_wireless_alarm_system_fuaa50000:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>wireless alarm system</t>
         </is>
       </c>
     </row>
@@ -3067,8 +3625,10 @@
       <c r="D81" t="n">
         <v>5.5</v>
       </c>
-      <c r="E81" t="n">
-        <v>3.1</v>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F81" t="inlineStr">
         <is>
@@ -3078,6 +3638,11 @@
       <c r="G81" t="inlineStr">
         <is>
           <t>cpe:2.3:o:simplisafe:simplisafe_ss3_firmware:1.4:*:*:*:*:*:*:*|cpe:2.3:h:simplisafe:simplisafe_ss3:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>simplisafe</t>
         </is>
       </c>
     </row>
@@ -3100,8 +3665,10 @@
       <c r="D82" t="n">
         <v>4.6</v>
       </c>
-      <c r="E82" t="n">
-        <v>3.1</v>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F82" t="inlineStr">
         <is>
@@ -3111,6 +3678,11 @@
       <c r="G82" t="inlineStr">
         <is>
           <t>cpe:2.3:o:simplisafe:ss3_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:simplisafe:ss3:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>simplisafe</t>
         </is>
       </c>
     </row>
@@ -3133,8 +3705,10 @@
       <c r="D83" t="n">
         <v>8.1</v>
       </c>
-      <c r="E83" t="n">
-        <v>3.1</v>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F83" t="inlineStr">
         <is>
@@ -3144,6 +3718,11 @@
       <c r="G83" t="inlineStr">
         <is>
           <t>cpe:2.3:o:abus:secvest_wireless_control_fube50001_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:abus:secvest_wireless_control_fube50001:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>wireless alarm system</t>
         </is>
       </c>
     </row>
@@ -3166,8 +3745,10 @@
       <c r="D84" t="n">
         <v>9.1</v>
       </c>
-      <c r="E84" t="n">
-        <v>3.1</v>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F84" t="inlineStr">
         <is>
@@ -3177,6 +3758,11 @@
       <c r="G84" t="inlineStr">
         <is>
           <t>cpe:2.3:o:abus:secvest_hybrid_fumo50110_firmware:-:*:*:*:*:*:*:*|cpe:2.3:h:abus:secvest_hybrid_fumo50110:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>alarm panel</t>
         </is>
       </c>
     </row>
@@ -3199,8 +3785,10 @@
       <c r="D85" t="n">
         <v>5.9</v>
       </c>
-      <c r="E85" t="n">
-        <v>3.1</v>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F85" t="inlineStr">
         <is>
@@ -3210,6 +3798,11 @@
       <c r="G85" t="inlineStr">
         <is>
           <t>cpe:2.3:o:fibaro:home_center_2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fibaro:home_center_2:-:*:*:*:*:*:*:*|cpe:2.3:o:fibaro:home_center_lite_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fibaro:home_center_lite:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>fibaro home center</t>
         </is>
       </c>
     </row>
@@ -3232,8 +3825,10 @@
       <c r="D86" t="n">
         <v>7.5</v>
       </c>
-      <c r="E86" t="n">
-        <v>3.1</v>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F86" t="inlineStr">
         <is>
@@ -3243,6 +3838,11 @@
       <c r="G86" t="inlineStr">
         <is>
           <t>cpe:2.3:o:fibaro:home_center_2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fibaro:home_center_2:-:*:*:*:*:*:*:*|cpe:2.3:o:fibaro:home_center_lite_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fibaro:home_center_lite:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>fibaro home center</t>
         </is>
       </c>
     </row>
@@ -3265,8 +3865,10 @@
       <c r="D87" t="n">
         <v>8.800000000000001</v>
       </c>
-      <c r="E87" t="n">
-        <v>3.1</v>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F87" t="inlineStr">
         <is>
@@ -3276,6 +3878,11 @@
       <c r="G87" t="inlineStr">
         <is>
           <t>cpe:2.3:o:fibaro:home_center_2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fibaro:home_center_2:-:*:*:*:*:*:*:*|cpe:2.3:o:fibaro:home_center_lite_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fibaro:home_center_lite:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>fibaro home center</t>
         </is>
       </c>
     </row>
@@ -3298,8 +3905,10 @@
       <c r="D88" t="n">
         <v>7.5</v>
       </c>
-      <c r="E88" t="n">
-        <v>3.1</v>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F88" t="inlineStr">
         <is>
@@ -3309,6 +3918,11 @@
       <c r="G88" t="inlineStr">
         <is>
           <t>cpe:2.3:o:fibaro:home_center_2_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fibaro:home_center_2:-:*:*:*:*:*:*:*|cpe:2.3:o:fibaro:home_center_lite_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:fibaro:home_center_lite:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>fibaro home center</t>
         </is>
       </c>
     </row>
@@ -3331,8 +3945,10 @@
       <c r="D89" t="n">
         <v>7.5</v>
       </c>
-      <c r="E89" t="n">
-        <v>3.1</v>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
@@ -3342,6 +3958,11 @@
       <c r="G89" t="inlineStr">
         <is>
           <t>cpe:2.3:o:abus:secvest_wireless_alarm_system_fuaa50000_firmware:3.01.17:*:*:*:*:*:*:*|cpe:2.3:h:abus:secvest_wireless_alarm_system_fuaa50000:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>wireless alarm system</t>
         </is>
       </c>
     </row>
@@ -3364,8 +3985,10 @@
       <c r="D90" t="n">
         <v>7.5</v>
       </c>
-      <c r="E90" t="n">
-        <v>3.1</v>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F90" t="inlineStr">
         <is>
@@ -3375,6 +3998,11 @@
       <c r="G90" t="inlineStr">
         <is>
           <t>cpe:2.3:a:hillrom:connex_central_station:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:connex_device_integration_suite_network_connectivity_engine:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:connex_integrated_wall_system:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:connex_spot_monitor:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:connex_vital_signs_monitor:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:service_monitor:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:service_tool:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:software_development_kit:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:spot_vital_signs_4400:*:*:*:*:-:*:*:*|cpe:2.3:a:hillrom:spot_vital_signs_4400:*:*:*:*:extended_care:*:*:*</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>central station</t>
         </is>
       </c>
     </row>
@@ -3397,8 +4025,10 @@
       <c r="D91" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E91" t="n">
-        <v>3.1</v>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F91" t="inlineStr">
         <is>
@@ -3408,6 +4038,11 @@
       <c r="G91" t="inlineStr">
         <is>
           <t>cpe:2.3:a:hillrom:connex_central_station:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:connex_device_integration_suite_network_connectivity_engine:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:connex_integrated_wall_system:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:connex_spot_monitor:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:connex_vital_signs_monitor:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:service_monitor:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:service_tool:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:software_development_kit:*:*:*:*:*:*:*:*|cpe:2.3:a:hillrom:spot_vital_signs_4400:*:*:*:*:-:*:*:*|cpe:2.3:a:hillrom:spot_vital_signs_4400:*:*:*:*:extended_care:*:*:*</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>central station</t>
         </is>
       </c>
     </row>
@@ -3430,8 +4065,10 @@
       <c r="D92" t="n">
         <v>10</v>
       </c>
-      <c r="E92" t="n">
-        <v>3.1</v>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F92" t="inlineStr">
         <is>
@@ -3441,6 +4078,11 @@
       <c r="G92" t="inlineStr">
         <is>
           <t>cpe:2.3:o:anker:eufy_homebase_2_firmware:2.1.6.9h:*:*:*:*:*:*:*|cpe:2.3:h:anker:eufy_homebase_2:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>eufy homebase</t>
         </is>
       </c>
     </row>
@@ -3463,8 +4105,10 @@
       <c r="D93" t="n">
         <v>10</v>
       </c>
-      <c r="E93" t="n">
-        <v>3.1</v>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F93" t="inlineStr">
         <is>
@@ -3474,6 +4118,11 @@
       <c r="G93" t="inlineStr">
         <is>
           <t>cpe:2.3:o:anker:eufy_homebase_2_firmware:2.1.6.9h:*:*:*:*:*:*:*|cpe:2.3:h:anker:eufy_homebase_2:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>eufy homebase</t>
         </is>
       </c>
     </row>
@@ -3496,8 +4145,10 @@
       <c r="D94" t="n">
         <v>9.9</v>
       </c>
-      <c r="E94" t="n">
-        <v>3.1</v>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F94" t="inlineStr">
         <is>
@@ -3507,6 +4158,11 @@
       <c r="G94" t="inlineStr">
         <is>
           <t>cpe:2.3:o:anker:eufy_homebase_2_firmware:2.1.6.9h:*:*:*:*:*:*:*|cpe:2.3:h:anker:eufy_homebase_2:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>eufy homebase</t>
         </is>
       </c>
     </row>
@@ -3529,8 +4185,10 @@
       <c r="D95" t="n">
         <v>7.5</v>
       </c>
-      <c r="E95" t="n">
-        <v>3.1</v>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F95" t="inlineStr">
         <is>
@@ -3540,6 +4198,11 @@
       <c r="G95" t="inlineStr">
         <is>
           <t>cpe:2.3:o:anker:eufy_homebase_2_firmware:2.1.6.9h:*:*:*:*:*:*:*|cpe:2.3:h:anker:eufy_homebase_2:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>eufy homebase</t>
         </is>
       </c>
     </row>
@@ -3562,8 +4225,10 @@
       <c r="D96" t="n">
         <v>6.8</v>
       </c>
-      <c r="E96" t="n">
-        <v>3.1</v>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F96" t="inlineStr">
         <is>
@@ -3573,6 +4238,11 @@
       <c r="G96" t="inlineStr">
         <is>
           <t>cpe:2.3:o:securitashome:securitashome_alarm_system_firmware:hpgw-g_0.0.2.23f_bg_u-itr-f1-bd_bl.a30.20181117:*:*:*:*:*:*:*|cpe:2.3:h:securitashome:securitashome_alarm_system:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>home alarm</t>
         </is>
       </c>
     </row>
@@ -3595,8 +4265,10 @@
       <c r="D97" t="n">
         <v>5.3</v>
       </c>
-      <c r="E97" t="n">
-        <v>3.1</v>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F97" t="inlineStr"/>
       <c r="G97" t="inlineStr">
@@ -3604,6 +4276,11 @@
           <t>cpe:2.3:o:securitashome:securitashome_alarm_system_firmware:hpgw-g_0.0.2.23f_bg_u-itr-f1-bd_bl.a30.20181117:*:*:*:*:*:*:*|cpe:2.3:h:securitashome:securitashome_alarm_system:-:*:*:*:*:*:*:*</t>
         </is>
       </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>home alarm</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3624,8 +4301,10 @@
       <c r="D98" t="n">
         <v>7.8</v>
       </c>
-      <c r="E98" t="n">
-        <v>3.1</v>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F98" t="inlineStr">
         <is>
@@ -3635,6 +4314,11 @@
       <c r="G98" t="inlineStr">
         <is>
           <t>cpe:2.3:o:goabode:iota_all-in-one_security_kit_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:goabode:iota_all-in-one_security_kit:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>abode iota</t>
         </is>
       </c>
     </row>
@@ -3657,8 +4341,10 @@
       <c r="D99" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E99" t="n">
-        <v>3.1</v>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
@@ -3668,6 +4354,11 @@
       <c r="G99" t="inlineStr">
         <is>
           <t>cpe:2.3:o:anker:eufy_homebase_2_firmware:2.1.6.9h:*:*:*:*:*:*:*|cpe:2.3:h:anker:eufy_homebase_2:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>eufy homebase</t>
         </is>
       </c>
     </row>
@@ -3690,8 +4381,10 @@
       <c r="D100" t="n">
         <v>8.1</v>
       </c>
-      <c r="E100" t="n">
-        <v>3.1</v>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F100" t="inlineStr">
         <is>
@@ -3701,6 +4394,11 @@
       <c r="G100" t="inlineStr">
         <is>
           <t>cpe:2.3:o:anker:eufy_homebase_2_firmware:2.1.6.9h:*:*:*:*:*:*:*|cpe:2.3:h:anker:eufy_homebase_2:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>eufy homebase</t>
         </is>
       </c>
     </row>
@@ -3723,8 +4421,10 @@
       <c r="D101" t="n">
         <v>9.800000000000001</v>
       </c>
-      <c r="E101" t="n">
-        <v>3.1</v>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F101" t="inlineStr">
         <is>
@@ -3734,6 +4434,11 @@
       <c r="G101" t="inlineStr">
         <is>
           <t>cpe:2.3:o:johnsoncontrols:qolsys_iq_panel_4_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:johnsoncontrols:qolsys_iq_panel_4:-:*:*:*:*:*:*:*|cpe:2.3:o:johnsoncontrols:qolsys_iq4_hub_firmware:*:*:*:*:*:*:*:*|cpe:2.3:h:johnsoncontrols:qolsys_iq4_hub:-:*:*:*:*:*:*:*</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>qolsys</t>
         </is>
       </c>
     </row>
@@ -3761,6 +4466,11 @@
         </is>
       </c>
       <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>monitoring station</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3786,6 +4496,11 @@
         </is>
       </c>
       <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>hubitat</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3806,8 +4521,10 @@
       <c r="D104" t="n">
         <v>7.7</v>
       </c>
-      <c r="E104" t="n">
-        <v>3.1</v>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>3.1</t>
+        </is>
       </c>
       <c r="F104" t="inlineStr">
         <is>
@@ -3815,6 +4532,11 @@
         </is>
       </c>
       <c r="G104" t="inlineStr"/>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>eufy homebase</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>